<commit_message>
add toast for CRUD operations, excel export for bangcongno
</commit_message>
<xml_diff>
--- a/public/lsx.xlsx
+++ b/public/lsx.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\diepm\Desktop\git\diepgia-management\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D7275DD-96B4-46C7-9223-39506847F908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C786CC80-ECFA-4E62-B5C7-0217490142BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14303" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -157,16 +157,16 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="thin">
+      <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -175,7 +175,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -201,29 +201,23 @@
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -506,32 +500,32 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.59765625" customWidth="1"/>
-    <col min="2" max="2" width="19.1328125" customWidth="1"/>
-    <col min="3" max="3" width="12.1328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.5703125" style="15" customWidth="1"/>
+    <col min="2" max="2" width="19.140625" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="17.25" x14ac:dyDescent="0.45">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="16"/>
-    </row>
-    <row r="2" spans="1:4" ht="17.25" x14ac:dyDescent="0.45">
-      <c r="A2" s="11" t="s">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="12"/>
+    </row>
+    <row r="2" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A2" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
       <c r="D2" s="1"/>
     </row>
-    <row r="3" spans="1:4" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A3" s="18" t="s">
+    <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="16" t="s">
         <v>8</v>
       </c>
       <c r="B3" s="2"/>
@@ -540,7 +534,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
@@ -548,7 +542,7 @@
       <c r="C4" s="7"/>
       <c r="D4" s="8"/>
     </row>
-    <row r="5" spans="1:4" ht="15.4" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
@@ -558,25 +552,25 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A6" s="17" t="s">
+    <row r="6" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="12"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="14"/>
-    </row>
-    <row r="7" spans="1:4" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A7" s="15" t="s">
+      <c r="B6" s="9"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="11"/>
+    </row>
+    <row r="7" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="15"/>
+      <c r="D7" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>